<commit_message>
Update New Relic market reports - 2026-10-11 15:13:55
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-11 19:49:58
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-12 13:17:48
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-12 20:41:48
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-13 06:08:32
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-13 16:09:24
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-13 17:20:20
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-14 17:43:09
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-15 01:17:26
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-15 15:26:27
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-15 19:36:38
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-16 15:05:37
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-16 19:10:44
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-17 13:29:41
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-17 16:46:36
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-17 18:58:22
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-17 21:17:20
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-17 23:41:27
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-18 07:39:15
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-18 12:21:13
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-18 16:17:57
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-18 19:09:24
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-21 15:50:55
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-21 19:51:20
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-22 12:44:17
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-23 10:49:43
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-23 19:41:57
</commit_message>
<xml_diff>
--- a/output/glo-de.xlsx
+++ b/output/glo-de.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">

</xml_diff>